<commit_message>
Separe les prix par famille et decrit chaque ecran au niveau du dashboard.
Les formules de tarification ne dependent plus de la categorie : champs dedies pour les accessoires, groupe Tarification lentilles + PEL, marque sur les lentilles.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Cahier de test/Cahier de test OctoPIM.xlsx
+++ b/docs/Cahier de test/Cahier de test OctoPIM.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1909,6 +1909,314 @@
       <c r="E57" t="inlineStr">
         <is>
           <t>L action est refusee ou absente. Le guide indique de contacter Alexis Beranger, administrateur de la solution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Affichage solaire</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Passer une monture optique en Solaire</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Miroir, Pola, Dégradé, teinte des verres et catégorie du verre apparaissent tout de suite, juste après Optique / Solaire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Teinte</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Ouvrir la teinte d'une monture solaire</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Les choix sont Brun, Gris, Rose, Vert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Style</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Ouvrir Style</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Les choix sont Classique, Fashion, Sport.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Profil</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Ouvrir Profil de caractère</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Les choix sont PFL0010 : Homme, PFL0030 : Mixte, PFL0020 : Femme, PFL0040 : Enfant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Matière</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Ouvrir Matière</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Métal est proposé. Metal ne l'est plus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Groupe de marchandise</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Monture optique, plastique, cerclée</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Le champ calculé vaut GM0040     Mont.Opt.Pl.Cerclées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Fournisseur</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Ouvrir la fiche Esprit 33513</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Nom du fournisseur = CHARMANT. Code fabricant = CHA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>IWI solaire</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Ouvrir une monture solaire plastique</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Type = B, prescription = 0, code douanier IWI = 9004109100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Code marquage</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Fiche Esprit 33513, couleur 545, calibre 48, nez 21</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Le code marquage vaut 33513 545 4821.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Attribut système</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Ouvrir un attribut système</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Le panneau est en consultation. Enregistrer n'est pas proposé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Attributs</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Quitter sans enregistrer</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Modifier le nom d'un attribut puis Annuler</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Une confirmation demande si l'on quitte sans enregistrer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Fiche</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Champ vide</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Ouvrir une fiche avec un champ de complétion vide</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Ce champ a un fond rose pâle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Sélection</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Cocher deux produits dans la liste puis ouvrir Exports</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Le compteur et le fichier ne contiennent que ces deux produits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Tout exporter</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Depuis une sélection, cliquer Tout exporter</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Le compteur revient à l'ensemble filtré.</t>
         </is>
       </c>
     </row>

</xml_diff>